<commit_message>
Skip classifier types with an empty notification list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/classifier.xlsx
+++ b/data/classifier.xlsx
@@ -2196,7 +2196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1133"/>
+  <dimension ref="A1:F1132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35804,7 +35804,7 @@
     <row r="1121">
       <c r="A1121" t="inlineStr">
         <is>
-          <t>23060001</t>
+          <t>24010000</t>
         </is>
       </c>
       <c r="B1121" t="inlineStr">
@@ -35814,23 +35814,27 @@
       </c>
       <c r="C1121" t="inlineStr">
         <is>
-          <t>Прочие происшествия (от 102)</t>
+          <t>БПЛА</t>
         </is>
       </c>
       <c r="D1121" t="inlineStr">
         <is>
-          <t>{"level1": "Прочие происшествия (от 102)", "level2": "Для простомотра операторов ОКр"}</t>
+          <t>{"level1": "готовят к запуску, летит"}</t>
         </is>
       </c>
       <c r="E1121" t="n">
-        <v>3</v>
-      </c>
-      <c r="F1121" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>S102,FSB,CODD,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB,MO_RHBZ</t>
+        </is>
+      </c>
     </row>
     <row r="1122">
       <c r="A1122" t="inlineStr">
         <is>
-          <t>24010000</t>
+          <t>24020000</t>
         </is>
       </c>
       <c r="B1122" t="inlineStr">
@@ -35840,27 +35844,27 @@
       </c>
       <c r="C1122" t="inlineStr">
         <is>
-          <t>БПЛА</t>
+          <t>БПЛА здание</t>
         </is>
       </c>
       <c r="D1122" t="inlineStr">
         <is>
-          <t>{"level1": "готовят к запуску, летит"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "жилой дом/административное здание"}</t>
         </is>
       </c>
       <c r="E1122" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F1122" t="inlineStr">
         <is>
-          <t>S102,FSB,CODD,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB,MO_RHBZ</t>
+          <t>S102,S104,FSB,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,DEP_GRSTROY,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,DGP,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1123">
       <c r="A1123" t="inlineStr">
         <is>
-          <t>24020000</t>
+          <t>24030000</t>
         </is>
       </c>
       <c r="B1123" t="inlineStr">
@@ -35870,27 +35874,27 @@
       </c>
       <c r="C1123" t="inlineStr">
         <is>
-          <t>БПЛА здание</t>
+          <t>БПЛА проезжая часть</t>
         </is>
       </c>
       <c r="D1123" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "жилой дом/административное здание"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "проезжая часть/тоннель/Мост/Эстакада/Подземный переход/Наземный переход"}</t>
         </is>
       </c>
       <c r="E1123" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F1123" t="inlineStr">
         <is>
-          <t>S102,S104,FSB,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,DEP_GRSTROY,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,DGP,CUKB</t>
+          <t>S102,S104,FSB,AVTODOR,GORMOST,CODD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1124">
       <c r="A1124" t="inlineStr">
         <is>
-          <t>24030000</t>
+          <t>24040000</t>
         </is>
       </c>
       <c r="B1124" t="inlineStr">
@@ -35900,12 +35904,12 @@
       </c>
       <c r="C1124" t="inlineStr">
         <is>
-          <t>БПЛА проезжая часть</t>
+          <t>БПЛА учебное заведение</t>
         </is>
       </c>
       <c r="D1124" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "проезжая часть/тоннель/Мост/Эстакада/Подземный переход/Наземный переход"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Учебное"}</t>
         </is>
       </c>
       <c r="E1124" t="n">
@@ -35913,14 +35917,14 @@
       </c>
       <c r="F1124" t="inlineStr">
         <is>
-          <t>S102,S104,FSB,AVTODOR,GORMOST,CODD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
+          <t>S102,S104,FSB,MOSVODOKANAL,ROSSETI,OEK,CODD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,DEP_OBR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
-          <t>24040000</t>
+          <t>24050000</t>
         </is>
       </c>
       <c r="B1125" t="inlineStr">
@@ -35930,27 +35934,27 @@
       </c>
       <c r="C1125" t="inlineStr">
         <is>
-          <t>БПЛА учебное заведение</t>
+          <t>БПЛА лечебное заведение</t>
         </is>
       </c>
       <c r="D1125" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Учебное"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Лечебное"}</t>
         </is>
       </c>
       <c r="E1125" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F1125" t="inlineStr">
         <is>
-          <t>S102,S104,FSB,MOSVODOKANAL,ROSSETI,OEK,CODD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,DEP_OBR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
+          <t>S102,S104,CEMP,FSB,MOSVODOKANAL,ROSSETI,OEK,CODD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1126">
       <c r="A1126" t="inlineStr">
         <is>
-          <t>24050000</t>
+          <t>24060000</t>
         </is>
       </c>
       <c r="B1126" t="inlineStr">
@@ -35960,27 +35964,27 @@
       </c>
       <c r="C1126" t="inlineStr">
         <is>
-          <t>БПЛА лечебное заведение</t>
+          <t>БПЛА коммуникации, объект связи</t>
         </is>
       </c>
       <c r="D1126" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Лечебное"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Коммуникации/Объект связи"}</t>
         </is>
       </c>
       <c r="E1126" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F1126" t="inlineStr">
         <is>
-          <t>S102,S104,CEMP,FSB,MOSVODOKANAL,ROSSETI,OEK,CODD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
+          <t>S102,S104,FSB,MGTS,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,MOSKOLLEKTOR,OATI,MOSVODOSTOK,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1127">
       <c r="A1127" t="inlineStr">
         <is>
-          <t>24060000</t>
+          <t>24070000</t>
         </is>
       </c>
       <c r="B1127" t="inlineStr">
@@ -35990,12 +35994,12 @@
       </c>
       <c r="C1127" t="inlineStr">
         <is>
-          <t>БПЛА коммуникации, объект связи</t>
+          <t>БПЛА Опасный объект, газопровод</t>
         </is>
       </c>
       <c r="D1127" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Коммуникации/Объект связи"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Опасный объект/Газопровод"}</t>
         </is>
       </c>
       <c r="E1127" t="n">
@@ -36003,14 +36007,14 @@
       </c>
       <c r="F1127" t="inlineStr">
         <is>
-          <t>S102,S104,FSB,MGTS,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,MOSKOLLEKTOR,OATI,MOSVODOSTOK,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
+          <t>S101,S102,S104,FSB,MGTS,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,MOSKOLLEKTOR,OATI,MOSVODOSTOK,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB,MO_RHBZ</t>
         </is>
       </c>
     </row>
     <row r="1128">
       <c r="A1128" t="inlineStr">
         <is>
-          <t>24070000</t>
+          <t>24080000</t>
         </is>
       </c>
       <c r="B1128" t="inlineStr">
@@ -36020,27 +36024,27 @@
       </c>
       <c r="C1128" t="inlineStr">
         <is>
-          <t>БПЛА Опасный объект, газопровод</t>
+          <t>БПЛА ЛЭП/Провода/контактная сеть</t>
         </is>
       </c>
       <c r="D1128" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Опасный объект/Газопровод"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "ЛЭП/Провода/ Контактная сеть"}</t>
         </is>
       </c>
       <c r="E1128" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F1128" t="inlineStr">
         <is>
-          <t>S101,S102,S104,FSB,MGTS,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,MOSKOLLEKTOR,OATI,MOSVODOSTOK,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB,MO_RHBZ</t>
+          <t>S102,S104,FSB,METRO,ROSSETI,OEK,CODD,RZD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1129">
       <c r="A1129" t="inlineStr">
         <is>
-          <t>24080000</t>
+          <t>24090000</t>
         </is>
       </c>
       <c r="B1129" t="inlineStr">
@@ -36050,27 +36054,27 @@
       </c>
       <c r="C1129" t="inlineStr">
         <is>
-          <t>БПЛА ЛЭП/Провода/контактная сеть</t>
+          <t>БПЛА Транспорный объект</t>
         </is>
       </c>
       <c r="D1129" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "ЛЭП/Провода/ Контактная сеть"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Транспортный объект"}</t>
         </is>
       </c>
       <c r="E1129" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F1129" t="inlineStr">
         <is>
-          <t>S102,S104,FSB,METRO,ROSSETI,OEK,CODD,RZD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
+          <t>S102,S104,FSB,MOSGORTRANS,MGTS,METRO,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,RZD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,ORG_PEREVOZOK,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1130">
       <c r="A1130" t="inlineStr">
         <is>
-          <t>24090000</t>
+          <t>24100000</t>
         </is>
       </c>
       <c r="B1130" t="inlineStr">
@@ -36080,27 +36084,27 @@
       </c>
       <c r="C1130" t="inlineStr">
         <is>
-          <t>БПЛА Транспорный объект</t>
+          <t>БПЛА Военный объект</t>
         </is>
       </c>
       <c r="D1130" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Транспортный объект"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Военный объект"}</t>
         </is>
       </c>
       <c r="E1130" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F1130" t="inlineStr">
         <is>
-          <t>S102,S104,FSB,MOSGORTRANS,MGTS,METRO,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,RZD,OATI,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,ORG_PEREVOZOK,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
+          <t>S102,S104,FSB,MGTS,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,OATI,MOSVODOSTOK,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
-          <t>24100000</t>
+          <t>24110000</t>
         </is>
       </c>
       <c r="B1131" t="inlineStr">
@@ -36110,27 +36114,27 @@
       </c>
       <c r="C1131" t="inlineStr">
         <is>
-          <t>БПЛА Военный объект</t>
+          <t>БПЛА Прочее</t>
         </is>
       </c>
       <c r="D1131" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Военный объект"}</t>
+          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Прочее"}</t>
         </is>
       </c>
       <c r="E1131" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F1131" t="inlineStr">
         <is>
-          <t>S102,S104,FSB,MGTS,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,OATI,MOSVODOSTOK,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
+          <t>S102,S104,FSB,MGTS,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,MOSKOLLEKTOR,OATI,MOSVODOSTOK,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
         </is>
       </c>
     </row>
     <row r="1132">
       <c r="A1132" t="inlineStr">
         <is>
-          <t>24110000</t>
+          <t>24120100</t>
         </is>
       </c>
       <c r="B1132" t="inlineStr">
@@ -36140,48 +36144,18 @@
       </c>
       <c r="C1132" t="inlineStr">
         <is>
-          <t>БПЛА Прочее</t>
+          <t>БПЛА Регион</t>
         </is>
       </c>
       <c r="D1132" t="inlineStr">
         <is>
-          <t>{"level1": "упал/ столкнулся, нет взрыва возгорания", "level2": "Прочее"}</t>
+          <t>{"level1": "летит, готовят к запуску,упал/ столкнулся, нет взрыва возгорания", "level2": "Регион"}</t>
         </is>
       </c>
       <c r="E1132" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F1132" t="inlineStr">
-        <is>
-          <t>S102,S104,FSB,MGTS,MOSVODOKANAL,MOEK,ROSSETI,OEK,CODD,MOSKOLLEKTOR,OATI,MOSVODOSTOK,ROSGVARDIA,DDS_DISTRICT,DDS_TINAO,CITYENERGO,RBIPK,MAYOR,KOMENDATURA,NTU,FSO,GUP_MSR,CUKB</t>
-        </is>
-      </c>
-    </row>
-    <row r="1133">
-      <c r="A1133" t="inlineStr">
-        <is>
-          <t>24120100</t>
-        </is>
-      </c>
-      <c r="B1133" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="C1133" t="inlineStr">
-        <is>
-          <t>БПЛА Регион</t>
-        </is>
-      </c>
-      <c r="D1133" t="inlineStr">
-        <is>
-          <t>{"level1": "летит, готовят к запуску,упал/ столкнулся, нет взрыва возгорания", "level2": "Регион"}</t>
-        </is>
-      </c>
-      <c r="E1133" t="n">
-        <v>4</v>
-      </c>
-      <c r="F1133" t="inlineStr">
         <is>
           <t>S102,FSB,CITYENERGO,MAYOR,NTU,FSO,GUP_MSR,CUKB,MO_RHBZ</t>
         </is>

</xml_diff>